<commit_message>
update notebook & files
</commit_message>
<xml_diff>
--- a/test_pubmed_200.xlsx
+++ b/test_pubmed_200.xlsx
@@ -669,12 +669,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>J F, 2023, F1000RES</t>
+          <t>Figueroa-Quiñones J, 2023, F1000RES</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>J F, 2023, F1000RES</t>
+          <t>Figueroa-Quiñones J, 2023, F1000RES</t>
         </is>
       </c>
     </row>
@@ -795,12 +795,12 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>BP d, 2026, INT J MENT HEALTH ADDICT</t>
+          <t>de Mattos B, 2026, INT J MENT HEALTH ADDICT</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>BP d, 2026, INT J MENT HEALTH ADDICT</t>
+          <t>de Mattos B, 2026, INT J MENT HEALTH ADDICT</t>
         </is>
       </c>
     </row>
@@ -921,12 +921,12 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>A K, 2026, J DIABETES SCI TECHNOL</t>
+          <t>Kuang A, 2026, J DIABETES SCI TECHNOL</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>A K, 2026, J DIABETES SCI TECHNOL</t>
+          <t>Kuang A, 2026, J DIABETES SCI TECHNOL</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1039,12 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>C M, 2025, SMALL STRUCT</t>
+          <t>Marsico C, 2025, SMALL STRUCT</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>C M, 2025, SMALL STRUCT</t>
+          <t>Marsico C, 2025, SMALL STRUCT</t>
         </is>
       </c>
     </row>
@@ -1165,12 +1165,12 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>K U, 2026, COMPUT MECH</t>
+          <t>Upadhyay K, 2026, COMPUT MECH</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>K U, 2026, COMPUT MECH</t>
+          <t>Upadhyay K, 2026, COMPUT MECH</t>
         </is>
       </c>
     </row>
@@ -1283,12 +1283,12 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Z Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhan Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>Z Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhan Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -1401,12 +1401,12 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Y X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xie Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>Y X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xie Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -1519,12 +1519,12 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>S S, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Sivarajkumar S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>S S, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Sivarajkumar S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -1637,12 +1637,12 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>M W, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Wang M, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>M W, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Wang M, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>QN N, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Nguyen Q, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>QN N, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Nguyen Q, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -1873,12 +1873,12 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>P Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhang P, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>P Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhang P, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -1991,12 +1991,12 @@
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>B H, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Hoang B, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>B H, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Hoang B, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -2109,12 +2109,12 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Z X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xiang Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>Z X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xiang Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -2227,12 +2227,12 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>D X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xu D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>D X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xu D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -2345,12 +2345,12 @@
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>TM Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhang T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>TM Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhang T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -2463,12 +2463,12 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>D L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Le D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>D L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Le D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>S Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhang S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>S Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhang S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>A M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Michelet A, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>A M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Michelet A, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -2817,12 +2817,12 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>X L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Luo X, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>X L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Luo X, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -2935,12 +2935,12 @@
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>Z X, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Xu Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>Z X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xu Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3053,12 +3053,12 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>X H, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Hao X, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>X H, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Hao X, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3171,12 +3171,12 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>W L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Lau W, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>W L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Lau W, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3289,12 +3289,12 @@
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>N K, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Khatwani N, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>N K, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Khatwani N, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3407,12 +3407,12 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>L W, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Wang L, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>L W, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Wang L, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3525,12 +3525,12 @@
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>F C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Chen F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>F C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Chen F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3643,12 +3643,12 @@
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Y J, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Jiang Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>Y J, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Jiang Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3761,12 +3761,12 @@
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>H R, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Rehana H, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>H R, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Rehana H, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3879,12 +3879,12 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>N K, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Kumar N, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>N K, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Kumar N, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -3997,12 +3997,12 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>X L, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Li X, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>X L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Li X, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -4115,12 +4115,12 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>GM S, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Schaeferle G, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>GM S, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Schaeferle G, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -4233,12 +4233,12 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Y H, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Hu Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>Y H, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Hu Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -4351,12 +4351,12 @@
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>X H, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>He X, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>X H, 2024, AMIA ANNU SYMP PROC</t>
+          <t>He X, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -4469,12 +4469,12 @@
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>D W, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Wattegama D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>D W, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Wattegama D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -4587,12 +4587,12 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>B M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Mao B, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>B M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Mao B, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -4705,12 +4705,12 @@
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>L A, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Aust L, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>L A, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Aust L, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -4823,12 +4823,12 @@
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>F R, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Rezvani F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>F R, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Rezvani F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -4941,12 +4941,12 @@
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Y L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Luo Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>Y L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Luo Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -5059,12 +5059,12 @@
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>SJ X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xie S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
-          <t>SJ X, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Xie S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -5177,12 +5177,12 @@
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>A N, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Nagori A, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>A N, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Nagori A, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -5295,12 +5295,12 @@
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>EK L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Lee E, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>EK L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Lee E, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -5413,12 +5413,12 @@
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>JW B, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Betts J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>JW B, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Betts J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -5531,12 +5531,12 @@
       </c>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>T O, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Osborne T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>T O, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Osborne T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -5649,12 +5649,12 @@
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t>Q Y, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Yang Q, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>Q Y, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Yang Q, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -5767,12 +5767,12 @@
       </c>
       <c r="Y45" t="inlineStr">
         <is>
-          <t>Y L, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Lee Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>Y L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Lee Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -5885,12 +5885,12 @@
       </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>J F, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Finkelstein J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
-          <t>J F, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Finkelstein J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6003,12 +6003,12 @@
       </c>
       <c r="Y47" t="inlineStr">
         <is>
-          <t>HY C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Chen H, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z47" t="inlineStr">
         <is>
-          <t>HY C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Chen H, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6121,12 +6121,12 @@
       </c>
       <c r="Y48" t="inlineStr">
         <is>
-          <t>S Y, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Yang S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>S Y, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Yang S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6239,12 +6239,12 @@
       </c>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>Z L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Li Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>Z L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Li Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6357,12 +6357,12 @@
       </c>
       <c r="Y50" t="inlineStr">
         <is>
-          <t>S P, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Peddireddy S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>S P, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Peddireddy S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6475,12 +6475,12 @@
       </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>TTK M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Munia T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z51" t="inlineStr">
         <is>
-          <t>TTK M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Munia T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6593,12 +6593,12 @@
       </c>
       <c r="Y52" t="inlineStr">
         <is>
-          <t>AF C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Catapano A, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>AF C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Catapano A, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6711,12 +6711,12 @@
       </c>
       <c r="Y53" t="inlineStr">
         <is>
-          <t>Y L, 2024, AMIA ANNU SYMP PROC-a-b</t>
+          <t>Li Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>Y L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Li Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6829,12 +6829,12 @@
       </c>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>AD M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Mullen A, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>AD M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Mullen A, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -6947,12 +6947,12 @@
       </c>
       <c r="Y55" t="inlineStr">
         <is>
-          <t>NC W, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Wan N, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z55" t="inlineStr">
         <is>
-          <t>NC W, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Wan N, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -7065,12 +7065,12 @@
       </c>
       <c r="Y56" t="inlineStr">
         <is>
-          <t>JB E, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Edgcomb J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z56" t="inlineStr">
         <is>
-          <t>JB E, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Edgcomb J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -7183,12 +7183,12 @@
       </c>
       <c r="Y57" t="inlineStr">
         <is>
-          <t>T Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhou T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
-          <t>T Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhou T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -7301,12 +7301,12 @@
       </c>
       <c r="Y58" t="inlineStr">
         <is>
-          <t>MRS Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zawad M, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t>MRS Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zawad M, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -7419,12 +7419,12 @@
       </c>
       <c r="Y59" t="inlineStr">
         <is>
-          <t>J C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Chan J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>J C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Chan J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -7537,12 +7537,12 @@
       </c>
       <c r="Y60" t="inlineStr">
         <is>
-          <t>Y J, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Ji Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z60" t="inlineStr">
         <is>
-          <t>Y J, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Ji Y, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -7655,12 +7655,12 @@
       </c>
       <c r="Y61" t="inlineStr">
         <is>
-          <t>Ç O, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Ogğuztüzün Ç, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z61" t="inlineStr">
         <is>
-          <t>Ç O, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Ogğuztüzün Ç, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -7773,12 +7773,12 @@
       </c>
       <c r="Y62" t="inlineStr">
         <is>
-          <t>KY C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Chen K, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z62" t="inlineStr">
         <is>
-          <t>KY C, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Chen K, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -7891,12 +7891,12 @@
       </c>
       <c r="Y63" t="inlineStr">
         <is>
-          <t>TL R, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Reynolds T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
-          <t>TL R, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Reynolds T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8009,12 +8009,12 @@
       </c>
       <c r="Y64" t="inlineStr">
         <is>
-          <t>FL Y, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Yeh F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z64" t="inlineStr">
         <is>
-          <t>FL Y, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Yeh F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8127,12 +8127,12 @@
       </c>
       <c r="Y65" t="inlineStr">
         <is>
-          <t>DW K, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Kim D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z65" t="inlineStr">
         <is>
-          <t>DW K, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Kim D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8245,12 +8245,12 @@
       </c>
       <c r="Y66" t="inlineStr">
         <is>
-          <t>P M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Meka P, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z66" t="inlineStr">
         <is>
-          <t>P M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Meka P, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8363,12 +8363,12 @@
       </c>
       <c r="Y67" t="inlineStr">
         <is>
-          <t>LA T, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Tang L, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z67" t="inlineStr">
         <is>
-          <t>LA T, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Tang L, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8481,12 +8481,12 @@
       </c>
       <c r="Y68" t="inlineStr">
         <is>
-          <t>H Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhang H, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z68" t="inlineStr">
         <is>
-          <t>H Z, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Zhang H, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8599,12 +8599,12 @@
       </c>
       <c r="Y69" t="inlineStr">
         <is>
-          <t>Z D, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Duan Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z69" t="inlineStr">
         <is>
-          <t>Z D, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Duan Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8717,12 +8717,12 @@
       </c>
       <c r="Y70" t="inlineStr">
         <is>
-          <t>SA P, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Pungitore S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z70" t="inlineStr">
         <is>
-          <t>SA P, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Pungitore S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8835,12 +8835,12 @@
       </c>
       <c r="Y71" t="inlineStr">
         <is>
-          <t>Z D, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Ding Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z71" t="inlineStr">
         <is>
-          <t>Z D, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Ding Z, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -8953,12 +8953,12 @@
       </c>
       <c r="Y72" t="inlineStr">
         <is>
-          <t>D L, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Lee D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z72" t="inlineStr">
         <is>
-          <t>D L, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Lee D, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -9071,12 +9071,12 @@
       </c>
       <c r="Y73" t="inlineStr">
         <is>
-          <t>S S, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Shahabi S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z73" t="inlineStr">
         <is>
-          <t>S S, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Shahabi S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -9189,12 +9189,12 @@
       </c>
       <c r="Y74" t="inlineStr">
         <is>
-          <t>T S, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Shi T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z74" t="inlineStr">
         <is>
-          <t>T S, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Shi T, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -9307,12 +9307,12 @@
       </c>
       <c r="Y75" t="inlineStr">
         <is>
-          <t>J P, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Pradeepkumar J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z75" t="inlineStr">
         <is>
-          <t>J P, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Pradeepkumar J, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -9425,12 +9425,12 @@
       </c>
       <c r="Y76" t="inlineStr">
         <is>
-          <t>F A, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Amrollahi F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z76" t="inlineStr">
         <is>
-          <t>F A, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Amrollahi F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -9543,12 +9543,12 @@
       </c>
       <c r="Y77" t="inlineStr">
         <is>
-          <t>F A, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Amrollahi F, 2024, AMIA ANNU SYMP PROC-a</t>
         </is>
       </c>
       <c r="Z77" t="inlineStr">
         <is>
-          <t>F A, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Amrollahi F, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -9661,12 +9661,12 @@
       </c>
       <c r="Y78" t="inlineStr">
         <is>
-          <t>M A, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Asare-Baiden M, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z78" t="inlineStr">
         <is>
-          <t>M A, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Asare-Baiden M, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -9779,12 +9779,12 @@
       </c>
       <c r="Y79" t="inlineStr">
         <is>
-          <t>S Y, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Yadav S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
       <c r="Z79" t="inlineStr">
         <is>
-          <t>S Y, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Yadav S, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -9897,12 +9897,12 @@
       </c>
       <c r="Y80" t="inlineStr">
         <is>
-          <t>P M, 2024, AMIA ANNU SYMP PROC-a</t>
+          <t>Meka P, 2024, AMIA ANNU SYMP PROC-a</t>
         </is>
       </c>
       <c r="Z80" t="inlineStr">
         <is>
-          <t>P M, 2024, AMIA ANNU SYMP PROC</t>
+          <t>Meka P, 2024, AMIA ANNU SYMP PROC</t>
         </is>
       </c>
     </row>
@@ -10011,12 +10011,12 @@
       </c>
       <c r="Y81" t="inlineStr">
         <is>
-          <t>A D, 2025, EXPERT SYST APPL</t>
+          <t>Dabouei A, 2025, EXPERT SYST APPL</t>
         </is>
       </c>
       <c r="Z81" t="inlineStr">
         <is>
-          <t>A D, 2025, EXPERT SYST APPL</t>
+          <t>Dabouei A, 2025, EXPERT SYST APPL</t>
         </is>
       </c>
     </row>
@@ -10137,12 +10137,12 @@
       </c>
       <c r="Y82" t="inlineStr">
         <is>
-          <t>S V, 2026, J INTELL MANUF</t>
+          <t>Vagenas S, 2026, J INTELL MANUF</t>
         </is>
       </c>
       <c r="Z82" t="inlineStr">
         <is>
-          <t>S V, 2026, J INTELL MANUF</t>
+          <t>Vagenas S, 2026, J INTELL MANUF</t>
         </is>
       </c>
     </row>
@@ -10255,12 +10255,12 @@
       </c>
       <c r="Y83" t="inlineStr">
         <is>
-          <t>S G, 2023, F1000RES</t>
+          <t>Goudarzi S, 2023, F1000RES</t>
         </is>
       </c>
       <c r="Z83" t="inlineStr">
         <is>
-          <t>S G, 2023, F1000RES</t>
+          <t>Goudarzi S, 2023, F1000RES</t>
         </is>
       </c>
     </row>
@@ -10381,12 +10381,12 @@
       </c>
       <c r="Y84" t="inlineStr">
         <is>
-          <t>F C, 2025, SPAN J PSYCHIATRY MENT HEALTH</t>
+          <t>Corponi F, 2025, SPAN J PSYCHIATRY MENT HEALTH</t>
         </is>
       </c>
       <c r="Z84" t="inlineStr">
         <is>
-          <t>F C, 2025, SPAN J PSYCHIATRY MENT HEALTH</t>
+          <t>Corponi F, 2025, SPAN J PSYCHIATRY MENT HEALTH</t>
         </is>
       </c>
     </row>
@@ -10503,12 +10503,12 @@
       </c>
       <c r="Y85" t="inlineStr">
         <is>
-          <t>L M, 2024, PROCEEDINGS (IEEE INT CONF BIOINFORMATICS BIOMED)</t>
+          <t>Miao L, 2024, PROCEEDINGS (IEEE INT CONF BIOINFORMATICS BIOMED)</t>
         </is>
       </c>
       <c r="Z85" t="inlineStr">
         <is>
-          <t>L M, 2024, PROCEEDINGS (IEEE INT CONF BIOINFORMATICS BIOMED)</t>
+          <t>Miao L, 2024, PROCEEDINGS (IEEE INT CONF BIOINFORMATICS BIOMED)</t>
         </is>
       </c>
     </row>
@@ -10617,12 +10617,12 @@
       </c>
       <c r="Y86" t="inlineStr">
         <is>
-          <t>D M, 2024, EMERG TRENDS DRUGS ADDICT HEALTH</t>
+          <t>Murthy D, 2024, EMERG TRENDS DRUGS ADDICT HEALTH</t>
         </is>
       </c>
       <c r="Z86" t="inlineStr">
         <is>
-          <t>D M, 2024, EMERG TRENDS DRUGS ADDICT HEALTH</t>
+          <t>Murthy D, 2024, EMERG TRENDS DRUGS ADDICT HEALTH</t>
         </is>
       </c>
     </row>
@@ -10743,12 +10743,12 @@
       </c>
       <c r="Y87" t="inlineStr">
         <is>
-          <t>Z J, 2025, JAACAP OPEN</t>
+          <t>Jiang Z, 2025, JAACAP OPEN</t>
         </is>
       </c>
       <c r="Z87" t="inlineStr">
         <is>
-          <t>Z J, 2025, JAACAP OPEN</t>
+          <t>Jiang Z, 2025, JAACAP OPEN</t>
         </is>
       </c>
     </row>
@@ -10865,12 +10865,12 @@
       </c>
       <c r="Y88" t="inlineStr">
         <is>
-          <t>S C, 2025, INDIAN J TUBERC</t>
+          <t>Chattoraj S, 2025, INDIAN J TUBERC</t>
         </is>
       </c>
       <c r="Z88" t="inlineStr">
         <is>
-          <t>S C, 2025, INDIAN J TUBERC</t>
+          <t>Chattoraj S, 2025, INDIAN J TUBERC</t>
         </is>
       </c>
     </row>
@@ -10991,12 +10991,12 @@
       </c>
       <c r="Y89" t="inlineStr">
         <is>
-          <t>RK P, 2025, MED J ARMED FORCES INDIA</t>
+          <t>Pathni R, 2025, MED J ARMED FORCES INDIA</t>
         </is>
       </c>
       <c r="Z89" t="inlineStr">
         <is>
-          <t>RK P, 2025, MED J ARMED FORCES INDIA</t>
+          <t>Pathni R, 2025, MED J ARMED FORCES INDIA</t>
         </is>
       </c>
     </row>
@@ -11109,12 +11109,12 @@
       </c>
       <c r="Y90" t="inlineStr">
         <is>
-          <t>J H, 2023, WELLCOME OPEN RES</t>
+          <t>Hastings J, 2023, WELLCOME OPEN RES</t>
         </is>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
-          <t>J H, 2023, WELLCOME OPEN RES</t>
+          <t>Hastings J, 2023, WELLCOME OPEN RES</t>
         </is>
       </c>
     </row>
@@ -11235,12 +11235,12 @@
       </c>
       <c r="Y91" t="inlineStr">
         <is>
-          <t>BH P, 2025, COMPUT METHODS BIOMECH BIOMED ENGIN</t>
+          <t>Prasetio B, 2025, COMPUT METHODS BIOMECH BIOMED ENGIN</t>
         </is>
       </c>
       <c r="Z91" t="inlineStr">
         <is>
-          <t>BH P, 2025, COMPUT METHODS BIOMECH BIOMED ENGIN</t>
+          <t>Prasetio B, 2025, COMPUT METHODS BIOMECH BIOMED ENGIN</t>
         </is>
       </c>
     </row>
@@ -11353,12 +11353,12 @@
       </c>
       <c r="Y92" t="inlineStr">
         <is>
-          <t>A A, 2024, F1000RES</t>
+          <t>Achir A, 2024, F1000RES</t>
         </is>
       </c>
       <c r="Z92" t="inlineStr">
         <is>
-          <t>A A, 2024, F1000RES</t>
+          <t>Achir A, 2024, F1000RES</t>
         </is>
       </c>
     </row>
@@ -11475,12 +11475,12 @@
       </c>
       <c r="Y93" t="inlineStr">
         <is>
-          <t>J M, 2024, ADV NEURAL INF PROCESS SYST</t>
+          <t>Miao J, 2024, ADV NEURAL INF PROCESS SYST</t>
         </is>
       </c>
       <c r="Z93" t="inlineStr">
         <is>
-          <t>J M, 2024, ADV NEURAL INF PROCESS SYST</t>
+          <t>Miao J, 2024, ADV NEURAL INF PROCESS SYST</t>
         </is>
       </c>
     </row>
@@ -11601,12 +11601,12 @@
       </c>
       <c r="Y94" t="inlineStr">
         <is>
-          <t>SA T, 2025, J NEUROL SURG B SKULL BASE</t>
+          <t>Tenhoeve S, 2025, J NEUROL SURG B SKULL BASE</t>
         </is>
       </c>
       <c r="Z94" t="inlineStr">
         <is>
-          <t>SA T, 2025, J NEUROL SURG B SKULL BASE</t>
+          <t>Tenhoeve S, 2025, J NEUROL SURG B SKULL BASE</t>
         </is>
       </c>
     </row>
@@ -11723,12 +11723,12 @@
       </c>
       <c r="Y95" t="inlineStr">
         <is>
-          <t>HI H, 2024, PROC INT CONF IMAGE PROC</t>
+          <t>Helvaci H, 2024, PROC INT CONF IMAGE PROC</t>
         </is>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
-          <t>HI H, 2024, PROC INT CONF IMAGE PROC</t>
+          <t>Helvaci H, 2024, PROC INT CONF IMAGE PROC</t>
         </is>
       </c>
     </row>
@@ -11841,12 +11841,12 @@
       </c>
       <c r="Y96" t="inlineStr">
         <is>
-          <t>A O, 2025, J ENG SCI MED DIAGN THER</t>
+          <t>Olapojoye A, 2025, J ENG SCI MED DIAGN THER</t>
         </is>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
-          <t>A O, 2025, J ENG SCI MED DIAGN THER</t>
+          <t>Olapojoye A, 2025, J ENG SCI MED DIAGN THER</t>
         </is>
       </c>
     </row>
@@ -11959,12 +11959,12 @@
       </c>
       <c r="Y97" t="inlineStr">
         <is>
-          <t>N B, 2024, BIOINFORMATICS</t>
+          <t>Brunn N, 2024, BIOINFORMATICS</t>
         </is>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
-          <t>N B, 2024, BIOINFORMATICS</t>
+          <t>Brunn N, 2024, BIOINFORMATICS</t>
         </is>
       </c>
     </row>
@@ -12085,12 +12085,12 @@
       </c>
       <c r="Y98" t="inlineStr">
         <is>
-          <t>S T, 2025, INDIAN J HEMATOL BLOOD TRANSFUS</t>
+          <t>Thusoo S, 2025, INDIAN J HEMATOL BLOOD TRANSFUS</t>
         </is>
       </c>
       <c r="Z98" t="inlineStr">
         <is>
-          <t>S T, 2025, INDIAN J HEMATOL BLOOD TRANSFUS</t>
+          <t>Thusoo S, 2025, INDIAN J HEMATOL BLOOD TRANSFUS</t>
         </is>
       </c>
     </row>
@@ -12211,12 +12211,12 @@
       </c>
       <c r="Y99" t="inlineStr">
         <is>
-          <t>J V, 2025, FLOW TURBUL COMBUST</t>
+          <t>Vasanth J, 2025, FLOW TURBUL COMBUST</t>
         </is>
       </c>
       <c r="Z99" t="inlineStr">
         <is>
-          <t>J V, 2025, FLOW TURBUL COMBUST</t>
+          <t>Vasanth J, 2025, FLOW TURBUL COMBUST</t>
         </is>
       </c>
     </row>
@@ -12333,12 +12333,12 @@
       </c>
       <c r="Y100" t="inlineStr">
         <is>
-          <t>A Z, 2025, RADIOL ADV</t>
+          <t>Zhou A, 2025, RADIOL ADV</t>
         </is>
       </c>
       <c r="Z100" t="inlineStr">
         <is>
-          <t>A Z, 2025, RADIOL ADV</t>
+          <t>Zhou A, 2025, RADIOL ADV</t>
         </is>
       </c>
     </row>
@@ -12459,12 +12459,12 @@
       </c>
       <c r="Y101" t="inlineStr">
         <is>
-          <t>ES J, 2025, IEEE SENS J</t>
+          <t>Jeon E, 2025, IEEE SENS J</t>
         </is>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
-          <t>ES J, 2025, IEEE SENS J</t>
+          <t>Jeon E, 2025, IEEE SENS J</t>
         </is>
       </c>
     </row>
@@ -12585,12 +12585,12 @@
       </c>
       <c r="Y102" t="inlineStr">
         <is>
-          <t>M L, 2024, J CURR OPHTHALMOL</t>
+          <t>Lu M, 2024, J CURR OPHTHALMOL</t>
         </is>
       </c>
       <c r="Z102" t="inlineStr">
         <is>
-          <t>M L, 2024, J CURR OPHTHALMOL</t>
+          <t>Lu M, 2024, J CURR OPHTHALMOL</t>
         </is>
       </c>
     </row>
@@ -12695,12 +12695,12 @@
       </c>
       <c r="Y103" t="inlineStr">
         <is>
-          <t>J W, 2024, BIORXIV</t>
+          <t>Woodard J, 2024, BIORXIV</t>
         </is>
       </c>
       <c r="Z103" t="inlineStr">
         <is>
-          <t>J W, 2024, BIORXIV</t>
+          <t>Woodard J, 2024, BIORXIV</t>
         </is>
       </c>
     </row>
@@ -12821,12 +12821,12 @@
       </c>
       <c r="Y104" t="inlineStr">
         <is>
-          <t>H F, 2025, J COMPUT BIOPHYS CHEM</t>
+          <t>Feng H, 2025, J COMPUT BIOPHYS CHEM</t>
         </is>
       </c>
       <c r="Z104" t="inlineStr">
         <is>
-          <t>H F, 2025, J COMPUT BIOPHYS CHEM</t>
+          <t>Feng H, 2025, J COMPUT BIOPHYS CHEM</t>
         </is>
       </c>
     </row>
@@ -12947,12 +12947,12 @@
       </c>
       <c r="Y105" t="inlineStr">
         <is>
-          <t>PJA K, 2025, STIGMA HEALTH</t>
+          <t>Kelly P, 2025, STIGMA HEALTH</t>
         </is>
       </c>
       <c r="Z105" t="inlineStr">
         <is>
-          <t>PJA K, 2025, STIGMA HEALTH</t>
+          <t>Kelly P, 2025, STIGMA HEALTH</t>
         </is>
       </c>
     </row>
@@ -13073,12 +13073,12 @@
       </c>
       <c r="Y106" t="inlineStr">
         <is>
-          <t>V M, 2025, BULL EARTHQ ENG</t>
+          <t>Macchiarulo V, 2025, BULL EARTHQ ENG</t>
         </is>
       </c>
       <c r="Z106" t="inlineStr">
         <is>
-          <t>V M, 2025, BULL EARTHQ ENG</t>
+          <t>Macchiarulo V, 2025, BULL EARTHQ ENG</t>
         </is>
       </c>
     </row>
@@ -13187,12 +13187,12 @@
       </c>
       <c r="Y107" t="inlineStr">
         <is>
-          <t>R J, 2024, COMPUT CARDIOL (2010)</t>
+          <t>Jin R, 2024, COMPUT CARDIOL (2010)</t>
         </is>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
-          <t>R J, 2024, COMPUT CARDIOL (2010)</t>
+          <t>Jin R, 2024, COMPUT CARDIOL (2010)</t>
         </is>
       </c>
     </row>
@@ -13313,12 +13313,12 @@
       </c>
       <c r="Y108" t="inlineStr">
         <is>
-          <t>G B, 2024, MACH LEARN</t>
+          <t>Bhusal G, 2024, MACH LEARN</t>
         </is>
       </c>
       <c r="Z108" t="inlineStr">
         <is>
-          <t>G B, 2024, MACH LEARN</t>
+          <t>Bhusal G, 2024, MACH LEARN</t>
         </is>
       </c>
     </row>
@@ -13439,12 +13439,12 @@
       </c>
       <c r="Y109" t="inlineStr">
         <is>
-          <t>AA T, 2024, NAT MACH INTELL</t>
+          <t>Trotsyuk A, 2024, NAT MACH INTELL</t>
         </is>
       </c>
       <c r="Z109" t="inlineStr">
         <is>
-          <t>AA T, 2024, NAT MACH INTELL</t>
+          <t>Trotsyuk A, 2024, NAT MACH INTELL</t>
         </is>
       </c>
     </row>
@@ -13549,12 +13549,12 @@
       </c>
       <c r="Y110" t="inlineStr">
         <is>
-          <t>X L, 2024, PSYCHOL METHODS</t>
+          <t>Liu X, 2024, PSYCHOL METHODS</t>
         </is>
       </c>
       <c r="Z110" t="inlineStr">
         <is>
-          <t>X L, 2024, PSYCHOL METHODS</t>
+          <t>Liu X, 2024, PSYCHOL METHODS</t>
         </is>
       </c>
     </row>
@@ -13675,12 +13675,12 @@
       </c>
       <c r="Y111" t="inlineStr">
         <is>
-          <t>JF L, 2025, INT J ARTIF INTELL EDUC</t>
+          <t>Lohmann J, 2025, INT J ARTIF INTELL EDUC</t>
         </is>
       </c>
       <c r="Z111" t="inlineStr">
         <is>
-          <t>JF L, 2025, INT J ARTIF INTELL EDUC</t>
+          <t>Lohmann J, 2025, INT J ARTIF INTELL EDUC</t>
         </is>
       </c>
     </row>
@@ -13801,12 +13801,12 @@
       </c>
       <c r="Y112" t="inlineStr">
         <is>
-          <t>D X, 2025, INT J DATA SCI ANAL</t>
+          <t>Xu D, 2025, INT J DATA SCI ANAL</t>
         </is>
       </c>
       <c r="Z112" t="inlineStr">
         <is>
-          <t>D X, 2025, INT J DATA SCI ANAL</t>
+          <t>Xu D, 2025, INT J DATA SCI ANAL</t>
         </is>
       </c>
     </row>
@@ -13923,12 +13923,12 @@
       </c>
       <c r="Y113" t="inlineStr">
         <is>
-          <t>D R, 2025, JCPP ADV</t>
+          <t>Rakesh D, 2025, JCPP ADV</t>
         </is>
       </c>
       <c r="Z113" t="inlineStr">
         <is>
-          <t>D R, 2025, JCPP ADV</t>
+          <t>Rakesh D, 2025, JCPP ADV</t>
         </is>
       </c>
     </row>
@@ -14041,12 +14041,12 @@
       </c>
       <c r="Y114" t="inlineStr">
         <is>
-          <t>W Z, 2024, FRONT DRUG SAF REGUL</t>
+          <t>Zou W, 2024, FRONT DRUG SAF REGUL</t>
         </is>
       </c>
       <c r="Z114" t="inlineStr">
         <is>
-          <t>W Z, 2024, FRONT DRUG SAF REGUL</t>
+          <t>Zou W, 2024, FRONT DRUG SAF REGUL</t>
         </is>
       </c>
     </row>
@@ -14163,12 +14163,12 @@
       </c>
       <c r="Y115" t="inlineStr">
         <is>
-          <t>A V, 2025, J ORTHOP</t>
+          <t>Velasquez Garcia A, 2025, J ORTHOP</t>
         </is>
       </c>
       <c r="Z115" t="inlineStr">
         <is>
-          <t>A V, 2025, J ORTHOP</t>
+          <t>Velasquez Garcia A, 2025, J ORTHOP</t>
         </is>
       </c>
     </row>
@@ -14285,12 +14285,12 @@
       </c>
       <c r="Y116" t="inlineStr">
         <is>
-          <t>B X, 2025, ADV PROTEIN CHEM STRUCT BIOL</t>
+          <t>Xu B, 2025, ADV PROTEIN CHEM STRUCT BIOL</t>
         </is>
       </c>
       <c r="Z116" t="inlineStr">
         <is>
-          <t>B X, 2025, ADV PROTEIN CHEM STRUCT BIOL</t>
+          <t>Xu B, 2025, ADV PROTEIN CHEM STRUCT BIOL</t>
         </is>
       </c>
     </row>
@@ -14407,12 +14407,12 @@
       </c>
       <c r="Y117" t="inlineStr">
         <is>
-          <t>H Y, 2025, ADV PROTEIN CHEM STRUCT BIOL</t>
+          <t>Yu H, 2025, ADV PROTEIN CHEM STRUCT BIOL</t>
         </is>
       </c>
       <c r="Z117" t="inlineStr">
         <is>
-          <t>H Y, 2025, ADV PROTEIN CHEM STRUCT BIOL</t>
+          <t>Yu H, 2025, ADV PROTEIN CHEM STRUCT BIOL</t>
         </is>
       </c>
     </row>
@@ -14529,12 +14529,12 @@
       </c>
       <c r="Y118" t="inlineStr">
         <is>
-          <t>L W, 2025, IEEE TRANS AUTOM SCI ENG</t>
+          <t>Wang L, 2025, IEEE TRANS AUTOM SCI ENG</t>
         </is>
       </c>
       <c r="Z118" t="inlineStr">
         <is>
-          <t>L W, 2025, IEEE TRANS AUTOM SCI ENG</t>
+          <t>Wang L, 2025, IEEE TRANS AUTOM SCI ENG</t>
         </is>
       </c>
     </row>
@@ -14655,12 +14655,12 @@
       </c>
       <c r="Y119" t="inlineStr">
         <is>
-          <t>N B, 2024, J DATA SCI</t>
+          <t>Bo N, 2024, J DATA SCI</t>
         </is>
       </c>
       <c r="Z119" t="inlineStr">
         <is>
-          <t>N B, 2024, J DATA SCI</t>
+          <t>Bo N, 2024, J DATA SCI</t>
         </is>
       </c>
     </row>
@@ -14777,12 +14777,12 @@
       </c>
       <c r="Y120" t="inlineStr">
         <is>
-          <t>N L, 2024, INTERSPEECH</t>
+          <t>Lin N, 2024, INTERSPEECH</t>
         </is>
       </c>
       <c r="Z120" t="inlineStr">
         <is>
-          <t>N L, 2024, INTERSPEECH</t>
+          <t>Lin N, 2024, INTERSPEECH</t>
         </is>
       </c>
     </row>
@@ -14903,12 +14903,12 @@
       </c>
       <c r="Y121" t="inlineStr">
         <is>
-          <t>JB E, 2025, JAACAP OPEN</t>
+          <t>Edgcomb J, 2025, JAACAP OPEN</t>
         </is>
       </c>
       <c r="Z121" t="inlineStr">
         <is>
-          <t>JB E, 2025, JAACAP OPEN</t>
+          <t>Edgcomb J, 2025, JAACAP OPEN</t>
         </is>
       </c>
     </row>
@@ -15021,12 +15021,12 @@
       </c>
       <c r="Y122" t="inlineStr">
         <is>
-          <t>A V, 2024, F1000RES</t>
+          <t>Valencia-Arias A, 2024, F1000RES</t>
         </is>
       </c>
       <c r="Z122" t="inlineStr">
         <is>
-          <t>A V, 2024, F1000RES</t>
+          <t>Valencia-Arias A, 2024, F1000RES</t>
         </is>
       </c>
     </row>
@@ -15131,12 +15131,12 @@
       </c>
       <c r="Y123" t="inlineStr">
         <is>
-          <t>Y L, 2024, STAT BIOSCI</t>
+          <t>Lu Y, 2024, STAT BIOSCI</t>
         </is>
       </c>
       <c r="Z123" t="inlineStr">
         <is>
-          <t>Y L, 2024, STAT BIOSCI</t>
+          <t>Lu Y, 2024, STAT BIOSCI</t>
         </is>
       </c>
     </row>
@@ -15245,12 +15245,12 @@
       </c>
       <c r="Y124" t="inlineStr">
         <is>
-          <t>T R, 2024, PROC IEEE INT SYMP APPL FERROELECTR</t>
+          <t>Roy T, 2024, PROC IEEE INT SYMP APPL FERROELECTR</t>
         </is>
       </c>
       <c r="Z124" t="inlineStr">
         <is>
-          <t>T R, 2024, PROC IEEE INT SYMP APPL FERROELECTR</t>
+          <t>Roy T, 2024, PROC IEEE INT SYMP APPL FERROELECTR</t>
         </is>
       </c>
     </row>
@@ -15367,12 +15367,12 @@
       </c>
       <c r="Y125" t="inlineStr">
         <is>
-          <t>L M, 2025, IEEE TRANS AUTOM SCI ENG</t>
+          <t>Mao L, 2025, IEEE TRANS AUTOM SCI ENG</t>
         </is>
       </c>
       <c r="Z125" t="inlineStr">
         <is>
-          <t>L M, 2025, IEEE TRANS AUTOM SCI ENG</t>
+          <t>Mao L, 2025, IEEE TRANS AUTOM SCI ENG</t>
         </is>
       </c>
     </row>
@@ -15493,12 +15493,12 @@
       </c>
       <c r="Y126" t="inlineStr">
         <is>
-          <t>A v, 2025, AI SOC</t>
+          <t>van Oosterzee A, 2025, AI SOC</t>
         </is>
       </c>
       <c r="Z126" t="inlineStr">
         <is>
-          <t>A v, 2025, AI SOC</t>
+          <t>van Oosterzee A, 2025, AI SOC</t>
         </is>
       </c>
     </row>
@@ -15619,12 +15619,12 @@
       </c>
       <c r="Y127" t="inlineStr">
         <is>
-          <t>BI T, 2025, IEEE TRANS MOL BIOL MULTISCALE COMMUN</t>
+          <t>Tumenbayar B, 2025, IEEE TRANS MOL BIOL MULTISCALE COMMUN</t>
         </is>
       </c>
       <c r="Z127" t="inlineStr">
         <is>
-          <t>BI T, 2025, IEEE TRANS MOL BIOL MULTISCALE COMMUN</t>
+          <t>Tumenbayar B, 2025, IEEE TRANS MOL BIOL MULTISCALE COMMUN</t>
         </is>
       </c>
     </row>
@@ -15737,12 +15737,12 @@
       </c>
       <c r="Y128" t="inlineStr">
         <is>
-          <t>SV F, 2024, GATES OPEN RES</t>
+          <t>Flanagan S, 2024, GATES OPEN RES</t>
         </is>
       </c>
       <c r="Z128" t="inlineStr">
         <is>
-          <t>SV F, 2024, GATES OPEN RES</t>
+          <t>Flanagan S, 2024, GATES OPEN RES</t>
         </is>
       </c>
     </row>
@@ -15859,12 +15859,12 @@
       </c>
       <c r="Y129" t="inlineStr">
         <is>
-          <t>K G, 2024, BIOMED IMAGE REGIST PROC</t>
+          <t>Gopinath K, 2024, BIOMED IMAGE REGIST PROC</t>
         </is>
       </c>
       <c r="Z129" t="inlineStr">
         <is>
-          <t>K G, 2024, BIOMED IMAGE REGIST PROC</t>
+          <t>Gopinath K, 2024, BIOMED IMAGE REGIST PROC</t>
         </is>
       </c>
     </row>
@@ -15969,12 +15969,12 @@
       </c>
       <c r="Y130" t="inlineStr">
         <is>
-          <t>S A, 2024, IISE TRANS</t>
+          <t>Afshar S, 2024, IISE TRANS</t>
         </is>
       </c>
       <c r="Z130" t="inlineStr">
         <is>
-          <t>S A, 2024, IISE TRANS</t>
+          <t>Afshar S, 2024, IISE TRANS</t>
         </is>
       </c>
     </row>
@@ -16095,12 +16095,12 @@
       </c>
       <c r="Y131" t="inlineStr">
         <is>
-          <t>R P, 2025, POLICE J</t>
+          <t>Phythian R, 2025, POLICE J</t>
         </is>
       </c>
       <c r="Z131" t="inlineStr">
         <is>
-          <t>R P, 2025, POLICE J</t>
+          <t>Phythian R, 2025, POLICE J</t>
         </is>
       </c>
     </row>
@@ -16221,12 +16221,12 @@
       </c>
       <c r="Y132" t="inlineStr">
         <is>
-          <t>A C, 2024, IFAC PAP ONLINE</t>
+          <t>Comas A, 2024, IFAC PAP ONLINE</t>
         </is>
       </c>
       <c r="Z132" t="inlineStr">
         <is>
-          <t>A C, 2024, IFAC PAP ONLINE</t>
+          <t>Comas A, 2024, IFAC PAP ONLINE</t>
         </is>
       </c>
     </row>
@@ -16343,12 +16343,12 @@
       </c>
       <c r="Y133" t="inlineStr">
         <is>
-          <t>H X, 2025, J ENVIRON SCI (CHINA)</t>
+          <t>Xu H, 2025, J ENVIRON SCI (CHINA)</t>
         </is>
       </c>
       <c r="Z133" t="inlineStr">
         <is>
-          <t>H X, 2025, J ENVIRON SCI (CHINA)</t>
+          <t>Xu H, 2025, J ENVIRON SCI (CHINA)</t>
         </is>
       </c>
     </row>
@@ -16465,12 +16465,12 @@
       </c>
       <c r="Y134" t="inlineStr">
         <is>
-          <t>L S, 2025, J ENVIRON SCI (CHINA)</t>
+          <t>Song L, 2025, J ENVIRON SCI (CHINA)</t>
         </is>
       </c>
       <c r="Z134" t="inlineStr">
         <is>
-          <t>L S, 2025, J ENVIRON SCI (CHINA)</t>
+          <t>Song L, 2025, J ENVIRON SCI (CHINA)</t>
         </is>
       </c>
     </row>
@@ -16579,12 +16579,12 @@
       </c>
       <c r="Y135" t="inlineStr">
         <is>
-          <t>Y Z, 2025, CURR OPIN SOLID STATE MATER SCI</t>
+          <t>Zheng Y, 2025, CURR OPIN SOLID STATE MATER SCI</t>
         </is>
       </c>
       <c r="Z135" t="inlineStr">
         <is>
-          <t>Y Z, 2025, CURR OPIN SOLID STATE MATER SCI</t>
+          <t>Zheng Y, 2025, CURR OPIN SOLID STATE MATER SCI</t>
         </is>
       </c>
     </row>
@@ -16697,12 +16697,12 @@
       </c>
       <c r="Y136" t="inlineStr">
         <is>
-          <t>R U, 2024, ADV PHOTONICS</t>
+          <t>Unni R, 2024, ADV PHOTONICS</t>
         </is>
       </c>
       <c r="Z136" t="inlineStr">
         <is>
-          <t>R U, 2024, ADV PHOTONICS</t>
+          <t>Unni R, 2024, ADV PHOTONICS</t>
         </is>
       </c>
     </row>
@@ -16815,12 +16815,12 @@
       </c>
       <c r="Y137" t="inlineStr">
         <is>
-          <t>YJ C, 2025, ADV SENS RES</t>
+          <t>Cheng Y, 2025, ADV SENS RES</t>
         </is>
       </c>
       <c r="Z137" t="inlineStr">
         <is>
-          <t>YJ C, 2025, ADV SENS RES</t>
+          <t>Cheng Y, 2025, ADV SENS RES</t>
         </is>
       </c>
     </row>
@@ -16941,12 +16941,12 @@
       </c>
       <c r="Y138" t="inlineStr">
         <is>
-          <t>M Ö, 2025, HEALTH SYST (BASINGSTOKE)</t>
+          <t>Özcan M, 2025, HEALTH SYST (BASINGSTOKE)</t>
         </is>
       </c>
       <c r="Z138" t="inlineStr">
         <is>
-          <t>M Ö, 2025, HEALTH SYST (BASINGSTOKE)</t>
+          <t>Özcan M, 2025, HEALTH SYST (BASINGSTOKE)</t>
         </is>
       </c>
     </row>
@@ -17067,12 +17067,12 @@
       </c>
       <c r="Y139" t="inlineStr">
         <is>
-          <t>SI B, 2024, CURR TRANSPLANT REP</t>
+          <t>Berchuck S, 2024, CURR TRANSPLANT REP</t>
         </is>
       </c>
       <c r="Z139" t="inlineStr">
         <is>
-          <t>SI B, 2024, CURR TRANSPLANT REP</t>
+          <t>Berchuck S, 2024, CURR TRANSPLANT REP</t>
         </is>
       </c>
     </row>
@@ -17189,12 +17189,12 @@
       </c>
       <c r="Y140" t="inlineStr">
         <is>
-          <t>Y H, 2025, J PHARM ANAL</t>
+          <t>Hong Y, 2025, J PHARM ANAL</t>
         </is>
       </c>
       <c r="Z140" t="inlineStr">
         <is>
-          <t>Y H, 2025, J PHARM ANAL</t>
+          <t>Hong Y, 2025, J PHARM ANAL</t>
         </is>
       </c>
     </row>
@@ -17307,12 +17307,12 @@
       </c>
       <c r="Y141" t="inlineStr">
         <is>
-          <t>D D, 2024, MATHEMATICS (BASEL)</t>
+          <t>Duong-Tran D, 2024, MATHEMATICS (BASEL)</t>
         </is>
       </c>
       <c r="Z141" t="inlineStr">
         <is>
-          <t>D D, 2024, MATHEMATICS (BASEL)</t>
+          <t>Duong-Tran D, 2024, MATHEMATICS (BASEL)</t>
         </is>
       </c>
     </row>
@@ -17425,12 +17425,12 @@
       </c>
       <c r="Y142" t="inlineStr">
         <is>
-          <t>B N, 2024, FRONT SYST BIOL</t>
+          <t>Noordijk B, 2024, FRONT SYST BIOL</t>
         </is>
       </c>
       <c r="Z142" t="inlineStr">
         <is>
-          <t>B N, 2024, FRONT SYST BIOL</t>
+          <t>Noordijk B, 2024, FRONT SYST BIOL</t>
         </is>
       </c>
     </row>
@@ -17543,12 +17543,12 @@
       </c>
       <c r="Y143" t="inlineStr">
         <is>
-          <t>N P, 2024, FRONT SYST BIOL</t>
+          <t>Paul N, 2024, FRONT SYST BIOL</t>
         </is>
       </c>
       <c r="Z143" t="inlineStr">
         <is>
-          <t>N P, 2024, FRONT SYST BIOL</t>
+          <t>Paul N, 2024, FRONT SYST BIOL</t>
         </is>
       </c>
     </row>
@@ -17657,12 +17657,12 @@
       </c>
       <c r="Y144" t="inlineStr">
         <is>
-          <t>A H, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Harvey A, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
       <c r="Z144" t="inlineStr">
         <is>
-          <t>A H, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Harvey A, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
     </row>
@@ -17771,12 +17771,12 @@
       </c>
       <c r="Y145" t="inlineStr">
         <is>
-          <t>A G, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Grecucci A, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
       <c r="Z145" t="inlineStr">
         <is>
-          <t>A G, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Grecucci A, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
     </row>
@@ -17885,12 +17885,12 @@
       </c>
       <c r="Y146" t="inlineStr">
         <is>
-          <t>M K, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Kolisnyk M, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
       <c r="Z146" t="inlineStr">
         <is>
-          <t>M K, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Kolisnyk M, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
     </row>
@@ -17999,12 +17999,12 @@
       </c>
       <c r="Y147" t="inlineStr">
         <is>
-          <t>M G, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Garcia M, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
       <c r="Z147" t="inlineStr">
         <is>
-          <t>M G, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Garcia M, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
     </row>
@@ -18113,12 +18113,12 @@
       </c>
       <c r="Y148" t="inlineStr">
         <is>
-          <t>LA W, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Wallenwein L, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
       <c r="Z148" t="inlineStr">
         <is>
-          <t>LA W, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Wallenwein L, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
     </row>
@@ -18227,12 +18227,12 @@
       </c>
       <c r="Y149" t="inlineStr">
         <is>
-          <t>N W, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Wulan N, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
       <c r="Z149" t="inlineStr">
         <is>
-          <t>N W, 2024, IMAGING NEUROSCI (CAMB)</t>
+          <t>Wulan N, 2024, IMAGING NEUROSCI (CAMB)</t>
         </is>
       </c>
     </row>
@@ -18345,12 +18345,12 @@
       </c>
       <c r="Y150" t="inlineStr">
         <is>
-          <t>AW L, 2025, CAN J STAT</t>
+          <t>Levis A, 2025, CAN J STAT</t>
         </is>
       </c>
       <c r="Z150" t="inlineStr">
         <is>
-          <t>AW L, 2025, CAN J STAT</t>
+          <t>Levis A, 2025, CAN J STAT</t>
         </is>
       </c>
     </row>
@@ -18463,12 +18463,12 @@
       </c>
       <c r="Y151" t="inlineStr">
         <is>
-          <t>PM S, 2024, WELLCOME OPEN RES</t>
+          <t>Schenk P, 2024, WELLCOME OPEN RES</t>
         </is>
       </c>
       <c r="Z151" t="inlineStr">
         <is>
-          <t>PM S, 2024, WELLCOME OPEN RES</t>
+          <t>Schenk P, 2024, WELLCOME OPEN RES</t>
         </is>
       </c>
     </row>
@@ -18581,12 +18581,12 @@
       </c>
       <c r="Y152" t="inlineStr">
         <is>
-          <t>R A, 2024, WELLCOME OPEN RES</t>
+          <t>Ahmad R, 2024, WELLCOME OPEN RES</t>
         </is>
       </c>
       <c r="Z152" t="inlineStr">
         <is>
-          <t>R A, 2024, WELLCOME OPEN RES</t>
+          <t>Ahmad R, 2024, WELLCOME OPEN RES</t>
         </is>
       </c>
     </row>
@@ -18699,12 +18699,12 @@
       </c>
       <c r="Y153" t="inlineStr">
         <is>
-          <t>GR N, 2024, AJO INT</t>
+          <t>Nahass G, 2024, AJO INT</t>
         </is>
       </c>
       <c r="Z153" t="inlineStr">
         <is>
-          <t>GR N, 2024, AJO INT</t>
+          <t>Nahass G, 2024, AJO INT</t>
         </is>
       </c>
     </row>
@@ -18817,12 +18817,12 @@
       </c>
       <c r="Y154" t="inlineStr">
         <is>
-          <t>LL G, 2024, F1000RES</t>
+          <t>González L, 2024, F1000RES</t>
         </is>
       </c>
       <c r="Z154" t="inlineStr">
         <is>
-          <t>LL G, 2024, F1000RES</t>
+          <t>González L, 2024, F1000RES</t>
         </is>
       </c>
     </row>
@@ -18939,12 +18939,12 @@
       </c>
       <c r="Y155" t="inlineStr">
         <is>
-          <t>SQ H, 2024, ZHONGHUA NAN KE XUE</t>
+          <t>Huang S, 2024, ZHONGHUA NAN KE XUE</t>
         </is>
       </c>
       <c r="Z155" t="inlineStr">
         <is>
-          <t>SQ H, 2024, ZHONGHUA NAN KE XUE</t>
+          <t>Huang S, 2024, ZHONGHUA NAN KE XUE</t>
         </is>
       </c>
     </row>
@@ -19065,12 +19065,12 @@
       </c>
       <c r="Y156" t="inlineStr">
         <is>
-          <t>M P, 2024, NEW BIOETH</t>
+          <t>Pruski M, 2024, NEW BIOETH</t>
         </is>
       </c>
       <c r="Z156" t="inlineStr">
         <is>
-          <t>M P, 2024, NEW BIOETH</t>
+          <t>Pruski M, 2024, NEW BIOETH</t>
         </is>
       </c>
     </row>
@@ -19183,12 +19183,12 @@
       </c>
       <c r="Y157" t="inlineStr">
         <is>
-          <t>F E, 2025, ADV SENS RES</t>
+          <t>Ebrahimi F, 2025, ADV SENS RES</t>
         </is>
       </c>
       <c r="Z157" t="inlineStr">
         <is>
-          <t>F E, 2025, ADV SENS RES</t>
+          <t>Ebrahimi F, 2025, ADV SENS RES</t>
         </is>
       </c>
     </row>
@@ -19297,12 +19297,12 @@
       </c>
       <c r="Y158" t="inlineStr">
         <is>
-          <t>J T, 2024, SMART HEALTH (AMST)</t>
+          <t>Tian J, 2024, SMART HEALTH (AMST)</t>
         </is>
       </c>
       <c r="Z158" t="inlineStr">
         <is>
-          <t>J T, 2024, SMART HEALTH (AMST)</t>
+          <t>Tian J, 2024, SMART HEALTH (AMST)</t>
         </is>
       </c>
     </row>
@@ -19423,12 +19423,12 @@
       </c>
       <c r="Y159" t="inlineStr">
         <is>
-          <t>LM O, 2025, CLIN PSYCHOL SCI</t>
+          <t>O'Reilly L, 2025, CLIN PSYCHOL SCI</t>
         </is>
       </c>
       <c r="Z159" t="inlineStr">
         <is>
-          <t>LM O, 2025, CLIN PSYCHOL SCI</t>
+          <t>O'Reilly L, 2025, CLIN PSYCHOL SCI</t>
         </is>
       </c>
     </row>
@@ -19549,12 +19549,12 @@
       </c>
       <c r="Y160" t="inlineStr">
         <is>
-          <t>J J, 2025, NANOPHOTONICS</t>
+          <t>Jeffet J, 2025, NANOPHOTONICS</t>
         </is>
       </c>
       <c r="Z160" t="inlineStr">
         <is>
-          <t>J J, 2025, NANOPHOTONICS</t>
+          <t>Jeffet J, 2025, NANOPHOTONICS</t>
         </is>
       </c>
     </row>
@@ -19671,12 +19671,12 @@
       </c>
       <c r="Y161" t="inlineStr">
         <is>
-          <t>A F, 2024, OPEN RESPIR ARCH</t>
+          <t>Fernández-Tena A, 2024, OPEN RESPIR ARCH</t>
         </is>
       </c>
       <c r="Z161" t="inlineStr">
         <is>
-          <t>A F, 2024, OPEN RESPIR ARCH</t>
+          <t>Fernández-Tena A, 2024, OPEN RESPIR ARCH</t>
         </is>
       </c>
     </row>
@@ -19793,12 +19793,12 @@
       </c>
       <c r="Y162" t="inlineStr">
         <is>
-          <t>J A, 2025, J AM STAT ASSOC</t>
+          <t>Agterberg J, 2025, J AM STAT ASSOC</t>
         </is>
       </c>
       <c r="Z162" t="inlineStr">
         <is>
-          <t>J A, 2025, J AM STAT ASSOC</t>
+          <t>Agterberg J, 2025, J AM STAT ASSOC</t>
         </is>
       </c>
     </row>
@@ -19915,12 +19915,12 @@
       </c>
       <c r="Y163" t="inlineStr">
         <is>
-          <t>P L, 2024, REP U S</t>
+          <t>Leandro La Rotta P, 2024, REP U S</t>
         </is>
       </c>
       <c r="Z163" t="inlineStr">
         <is>
-          <t>P L, 2024, REP U S</t>
+          <t>Leandro La Rotta P, 2024, REP U S</t>
         </is>
       </c>
     </row>
@@ -20041,12 +20041,12 @@
       </c>
       <c r="Y164" t="inlineStr">
         <is>
-          <t>FO d, 2025, IEEE TRANS EVOL COMPUT</t>
+          <t>de Franca F, 2025, IEEE TRANS EVOL COMPUT</t>
         </is>
       </c>
       <c r="Z164" t="inlineStr">
         <is>
-          <t>FO d, 2025, IEEE TRANS EVOL COMPUT</t>
+          <t>de Franca F, 2025, IEEE TRANS EVOL COMPUT</t>
         </is>
       </c>
     </row>
@@ -20159,12 +20159,12 @@
       </c>
       <c r="Y165" t="inlineStr">
         <is>
-          <t>HN K, 2024, REPORTS (MDPI)</t>
+          <t>Kılıc H, 2024, REPORTS (MDPI)</t>
         </is>
       </c>
       <c r="Z165" t="inlineStr">
         <is>
-          <t>HN K, 2024, REPORTS (MDPI)</t>
+          <t>Kılıc H, 2024, REPORTS (MDPI)</t>
         </is>
       </c>
     </row>
@@ -20285,12 +20285,12 @@
       </c>
       <c r="Y166" t="inlineStr">
         <is>
-          <t>A K, 2024, MUSCLES</t>
+          <t>Kekelekis A, 2024, MUSCLES</t>
         </is>
       </c>
       <c r="Z166" t="inlineStr">
         <is>
-          <t>A K, 2024, MUSCLES</t>
+          <t>Kekelekis A, 2024, MUSCLES</t>
         </is>
       </c>
     </row>
@@ -20411,12 +20411,12 @@
       </c>
       <c r="Y167" t="inlineStr">
         <is>
-          <t>L M, 2024, IEEE TRANS AUTOM SCI ENG</t>
+          <t>Mao L, 2024, IEEE TRANS AUTOM SCI ENG</t>
         </is>
       </c>
       <c r="Z167" t="inlineStr">
         <is>
-          <t>L M, 2024, IEEE TRANS AUTOM SCI ENG</t>
+          <t>Mao L, 2024, IEEE TRANS AUTOM SCI ENG</t>
         </is>
       </c>
     </row>
@@ -20659,12 +20659,12 @@
       </c>
       <c r="Y169" t="inlineStr">
         <is>
-          <t>X H, 2024, NANO RES</t>
+          <t>Hou X, 2024, NANO RES</t>
         </is>
       </c>
       <c r="Z169" t="inlineStr">
         <is>
-          <t>X H, 2024, NANO RES</t>
+          <t>Hou X, 2024, NANO RES</t>
         </is>
       </c>
     </row>
@@ -20785,12 +20785,12 @@
       </c>
       <c r="Y170" t="inlineStr">
         <is>
-          <t>A P, 2025, NEURAL COMPUT APPL</t>
+          <t>Penzkofer A, 2025, NEURAL COMPUT APPL</t>
         </is>
       </c>
       <c r="Z170" t="inlineStr">
         <is>
-          <t>A P, 2025, NEURAL COMPUT APPL</t>
+          <t>Penzkofer A, 2025, NEURAL COMPUT APPL</t>
         </is>
       </c>
     </row>
@@ -20911,12 +20911,12 @@
       </c>
       <c r="Y171" t="inlineStr">
         <is>
-          <t>AW M, 2024, INT J STAT APPL MATH</t>
+          <t>Masinde A, 2024, INT J STAT APPL MATH</t>
         </is>
       </c>
       <c r="Z171" t="inlineStr">
         <is>
-          <t>AW M, 2024, INT J STAT APPL MATH</t>
+          <t>Masinde A, 2024, INT J STAT APPL MATH</t>
         </is>
       </c>
     </row>
@@ -21025,12 +21025,12 @@
       </c>
       <c r="Y172" t="inlineStr">
         <is>
-          <t>A L, 2024, MICROCHEM J</t>
+          <t>Laliwala A, 2024, MICROCHEM J</t>
         </is>
       </c>
       <c r="Z172" t="inlineStr">
         <is>
-          <t>A L, 2024, MICROCHEM J</t>
+          <t>Laliwala A, 2024, MICROCHEM J</t>
         </is>
       </c>
     </row>
@@ -21147,12 +21147,12 @@
       </c>
       <c r="Y173" t="inlineStr">
         <is>
-          <t>YL L, 2025, ADV INTELL SYST</t>
+          <t>Li Y, 2025, ADV INTELL SYST</t>
         </is>
       </c>
       <c r="Z173" t="inlineStr">
         <is>
-          <t>YL L, 2025, ADV INTELL SYST</t>
+          <t>Li Y, 2025, ADV INTELL SYST</t>
         </is>
       </c>
     </row>
@@ -21269,12 +21269,12 @@
       </c>
       <c r="Y174" t="inlineStr">
         <is>
-          <t>S H, 2024, EWHA MED J</t>
+          <t>Huh S, 2024, EWHA MED J</t>
         </is>
       </c>
       <c r="Z174" t="inlineStr">
         <is>
-          <t>S H, 2024, EWHA MED J</t>
+          <t>Huh S, 2024, EWHA MED J</t>
         </is>
       </c>
     </row>
@@ -21395,12 +21395,12 @@
       </c>
       <c r="Y175" t="inlineStr">
         <is>
-          <t>NJ W, 2025, MED J ARMED FORCES INDIA</t>
+          <t>Waghray N, 2025, MED J ARMED FORCES INDIA</t>
         </is>
       </c>
       <c r="Z175" t="inlineStr">
         <is>
-          <t>NJ W, 2025, MED J ARMED FORCES INDIA</t>
+          <t>Waghray N, 2025, MED J ARMED FORCES INDIA</t>
         </is>
       </c>
     </row>
@@ -21505,12 +21505,12 @@
       </c>
       <c r="Y176" t="inlineStr">
         <is>
-          <t>K T, 2024, J R STAT SOC SER A STAT SOC</t>
+          <t>Takatsu K, 2024, J R STAT SOC SER A STAT SOC</t>
         </is>
       </c>
       <c r="Z176" t="inlineStr">
         <is>
-          <t>K T, 2024, J R STAT SOC SER A STAT SOC</t>
+          <t>Takatsu K, 2024, J R STAT SOC SER A STAT SOC</t>
         </is>
       </c>
     </row>
@@ -21615,12 +21615,12 @@
       </c>
       <c r="Y177" t="inlineStr">
         <is>
-          <t>E H, 2024, BIORXIV</t>
+          <t>Hasanaj E, 2024, BIORXIV</t>
         </is>
       </c>
       <c r="Z177" t="inlineStr">
         <is>
-          <t>E H, 2024, BIORXIV</t>
+          <t>Hasanaj E, 2024, BIORXIV</t>
         </is>
       </c>
     </row>
@@ -21737,12 +21737,12 @@
       </c>
       <c r="Y178" t="inlineStr">
         <is>
-          <t>K C, 2025, IEEE OPEN J ENG MED BIOL</t>
+          <t>Chansaengsri K, 2025, IEEE OPEN J ENG MED BIOL</t>
         </is>
       </c>
       <c r="Z178" t="inlineStr">
         <is>
-          <t>K C, 2025, IEEE OPEN J ENG MED BIOL</t>
+          <t>Chansaengsri K, 2025, IEEE OPEN J ENG MED BIOL</t>
         </is>
       </c>
     </row>
@@ -21855,12 +21855,12 @@
       </c>
       <c r="Y179" t="inlineStr">
         <is>
-          <t>Y L, 2024, NEUROSCI APPL</t>
+          <t>Li Y, 2024, NEUROSCI APPL</t>
         </is>
       </c>
       <c r="Z179" t="inlineStr">
         <is>
-          <t>Y L, 2024, NEUROSCI APPL</t>
+          <t>Li Y, 2024, NEUROSCI APPL</t>
         </is>
       </c>
     </row>
@@ -21973,12 +21973,12 @@
       </c>
       <c r="Y180" t="inlineStr">
         <is>
-          <t>TH M, 2024, J MOOD ANXIETY DISORD</t>
+          <t>McCoy T, 2024, J MOOD ANXIETY DISORD</t>
         </is>
       </c>
       <c r="Z180" t="inlineStr">
         <is>
-          <t>TH M, 2024, J MOOD ANXIETY DISORD</t>
+          <t>McCoy T, 2024, J MOOD ANXIETY DISORD</t>
         </is>
       </c>
     </row>
@@ -22091,12 +22091,12 @@
       </c>
       <c r="Y181" t="inlineStr">
         <is>
-          <t>BA Z, 2024, J MOOD ANXIETY DISORD</t>
+          <t>Zaboski B, 2024, J MOOD ANXIETY DISORD</t>
         </is>
       </c>
       <c r="Z181" t="inlineStr">
         <is>
-          <t>BA Z, 2024, J MOOD ANXIETY DISORD</t>
+          <t>Zaboski B, 2024, J MOOD ANXIETY DISORD</t>
         </is>
       </c>
     </row>
@@ -22209,12 +22209,12 @@
       </c>
       <c r="Y182" t="inlineStr">
         <is>
-          <t>A K, 2025, NEUROSCI APPL</t>
+          <t>Khuntia A, 2025, NEUROSCI APPL</t>
         </is>
       </c>
       <c r="Z182" t="inlineStr">
         <is>
-          <t>A K, 2025, NEUROSCI APPL</t>
+          <t>Khuntia A, 2025, NEUROSCI APPL</t>
         </is>
       </c>
     </row>
@@ -22327,12 +22327,12 @@
       </c>
       <c r="Y183" t="inlineStr">
         <is>
-          <t>C K, 2023, F1000RES</t>
+          <t>Khew C, 2023, F1000RES</t>
         </is>
       </c>
       <c r="Z183" t="inlineStr">
         <is>
-          <t>C K, 2023, F1000RES</t>
+          <t>Khew C, 2023, F1000RES</t>
         </is>
       </c>
     </row>
@@ -22449,12 +22449,12 @@
       </c>
       <c r="Y184" t="inlineStr">
         <is>
-          <t>CL O, 2024, AFR J LAB MED</t>
+          <t>Obi C, 2024, AFR J LAB MED</t>
         </is>
       </c>
       <c r="Z184" t="inlineStr">
         <is>
-          <t>CL O, 2024, AFR J LAB MED</t>
+          <t>Obi C, 2024, AFR J LAB MED</t>
         </is>
       </c>
     </row>
@@ -22571,12 +22571,12 @@
       </c>
       <c r="Y185" t="inlineStr">
         <is>
-          <t>S Y, 2025, ILIVER</t>
+          <t>Yu S, 2025, ILIVER</t>
         </is>
       </c>
       <c r="Z185" t="inlineStr">
         <is>
-          <t>S Y, 2025, ILIVER</t>
+          <t>Yu S, 2025, ILIVER</t>
         </is>
       </c>
     </row>
@@ -22681,12 +22681,12 @@
       </c>
       <c r="Y186" t="inlineStr">
         <is>
-          <t>GV K, 2024, BIORXIV</t>
+          <t>Kumar G, 2024, BIORXIV</t>
         </is>
       </c>
       <c r="Z186" t="inlineStr">
         <is>
-          <t>GV K, 2024, BIORXIV</t>
+          <t>Kumar G, 2024, BIORXIV</t>
         </is>
       </c>
     </row>
@@ -22803,12 +22803,12 @@
       </c>
       <c r="Y187" t="inlineStr">
         <is>
-          <t>X W, 2024, ILIVER</t>
+          <t>Wu X, 2024, ILIVER</t>
         </is>
       </c>
       <c r="Z187" t="inlineStr">
         <is>
-          <t>X W, 2024, ILIVER</t>
+          <t>Wu X, 2024, ILIVER</t>
         </is>
       </c>
     </row>
@@ -22925,12 +22925,12 @@
       </c>
       <c r="Y188" t="inlineStr">
         <is>
-          <t>L Z, 2025, SMART MOL</t>
+          <t>Zhao L, 2025, SMART MOL</t>
         </is>
       </c>
       <c r="Z188" t="inlineStr">
         <is>
-          <t>L Z, 2025, SMART MOL</t>
+          <t>Zhao L, 2025, SMART MOL</t>
         </is>
       </c>
     </row>
@@ -23051,12 +23051,12 @@
       </c>
       <c r="Y189" t="inlineStr">
         <is>
-          <t>SJ M, 2025, MATERN FETAL MED</t>
+          <t>Mathewlynn S, 2025, MATERN FETAL MED</t>
         </is>
       </c>
       <c r="Z189" t="inlineStr">
         <is>
-          <t>SJ M, 2025, MATERN FETAL MED</t>
+          <t>Mathewlynn S, 2025, MATERN FETAL MED</t>
         </is>
       </c>
     </row>
@@ -23173,12 +23173,12 @@
       </c>
       <c r="Y190" t="inlineStr">
         <is>
-          <t>K K, 2024, NPJ IMAGING</t>
+          <t>Kim K, 2024, NPJ IMAGING</t>
         </is>
       </c>
       <c r="Z190" t="inlineStr">
         <is>
-          <t>K K, 2024, NPJ IMAGING</t>
+          <t>Kim K, 2024, NPJ IMAGING</t>
         </is>
       </c>
     </row>
@@ -23295,12 +23295,12 @@
       </c>
       <c r="Y191" t="inlineStr">
         <is>
-          <t>S F, 2024, NPJ IMAGING</t>
+          <t>Fleig S, 2024, NPJ IMAGING</t>
         </is>
       </c>
       <c r="Z191" t="inlineStr">
         <is>
-          <t>S F, 2024, NPJ IMAGING</t>
+          <t>Fleig S, 2024, NPJ IMAGING</t>
         </is>
       </c>
     </row>
@@ -23417,12 +23417,12 @@
       </c>
       <c r="Y192" t="inlineStr">
         <is>
-          <t>A S, 2024, NPJ IMAGING</t>
+          <t>Shankar A, 2024, NPJ IMAGING</t>
         </is>
       </c>
       <c r="Z192" t="inlineStr">
         <is>
-          <t>A S, 2024, NPJ IMAGING</t>
+          <t>Shankar A, 2024, NPJ IMAGING</t>
         </is>
       </c>
     </row>
@@ -23539,12 +23539,12 @@
       </c>
       <c r="Y193" t="inlineStr">
         <is>
-          <t>L K, 2025, J ENVIRON SCI (CHINA)</t>
+          <t>Kuang L, 2025, J ENVIRON SCI (CHINA)</t>
         </is>
       </c>
       <c r="Z193" t="inlineStr">
         <is>
-          <t>L K, 2025, J ENVIRON SCI (CHINA)</t>
+          <t>Kuang L, 2025, J ENVIRON SCI (CHINA)</t>
         </is>
       </c>
     </row>
@@ -23657,12 +23657,12 @@
       </c>
       <c r="Y194" t="inlineStr">
         <is>
-          <t>T K, 2024, F1000RES</t>
+          <t>Katongtung T, 2024, F1000RES</t>
         </is>
       </c>
       <c r="Z194" t="inlineStr">
         <is>
-          <t>T K, 2024, F1000RES</t>
+          <t>Katongtung T, 2024, F1000RES</t>
         </is>
       </c>
     </row>
@@ -23775,12 +23775,12 @@
       </c>
       <c r="Y195" t="inlineStr">
         <is>
-          <t>T C, 2024, PROC MACH LEARN RES</t>
+          <t>Chang T, 2024, PROC MACH LEARN RES</t>
         </is>
       </c>
       <c r="Z195" t="inlineStr">
         <is>
-          <t>T C, 2024, PROC MACH LEARN RES</t>
+          <t>Chang T, 2024, PROC MACH LEARN RES</t>
         </is>
       </c>
     </row>
@@ -23897,12 +23897,12 @@
       </c>
       <c r="Y196" t="inlineStr">
         <is>
-          <t>G Y, 2024, NEUROIMAGE REP</t>
+          <t>Yang G, 2024, NEUROIMAGE REP</t>
         </is>
       </c>
       <c r="Z196" t="inlineStr">
         <is>
-          <t>G Y, 2024, NEUROIMAGE REP</t>
+          <t>Yang G, 2024, NEUROIMAGE REP</t>
         </is>
       </c>
     </row>
@@ -24019,12 +24019,12 @@
       </c>
       <c r="Y197" t="inlineStr">
         <is>
-          <t>R P, 2024, NEUROIMAGE REP</t>
+          <t>Poceviciute R, 2024, NEUROIMAGE REP</t>
         </is>
       </c>
       <c r="Z197" t="inlineStr">
         <is>
-          <t>R P, 2024, NEUROIMAGE REP</t>
+          <t>Poceviciute R, 2024, NEUROIMAGE REP</t>
         </is>
       </c>
     </row>
@@ -24145,12 +24145,12 @@
       </c>
       <c r="Y198" t="inlineStr">
         <is>
-          <t>AJ N, 2025, GERONTOLOGY</t>
+          <t>Nygård A, 2025, GERONTOLOGY</t>
         </is>
       </c>
       <c r="Z198" t="inlineStr">
         <is>
-          <t>AJ N, 2025, GERONTOLOGY</t>
+          <t>Nygård A, 2025, GERONTOLOGY</t>
         </is>
       </c>
     </row>
@@ -24271,12 +24271,12 @@
       </c>
       <c r="Y199" t="inlineStr">
         <is>
-          <t>M R, 2025, NAT REV ELECTR ENG</t>
+          <t>Ramezani M, 2025, NAT REV ELECTR ENG</t>
         </is>
       </c>
       <c r="Z199" t="inlineStr">
         <is>
-          <t>M R, 2025, NAT REV ELECTR ENG</t>
+          <t>Ramezani M, 2025, NAT REV ELECTR ENG</t>
         </is>
       </c>
     </row>
@@ -24397,12 +24397,12 @@
       </c>
       <c r="Y200" t="inlineStr">
         <is>
-          <t>D H, 2025, J CUTAN MED SURG</t>
+          <t>Hollman D, 2025, J CUTAN MED SURG</t>
         </is>
       </c>
       <c r="Z200" t="inlineStr">
         <is>
-          <t>D H, 2025, J CUTAN MED SURG</t>
+          <t>Hollman D, 2025, J CUTAN MED SURG</t>
         </is>
       </c>
     </row>
@@ -24523,12 +24523,12 @@
       </c>
       <c r="Y201" t="inlineStr">
         <is>
-          <t>R S, 2025, J AM STAT ASSOC</t>
+          <t>Sun R, 2025, J AM STAT ASSOC</t>
         </is>
       </c>
       <c r="Z201" t="inlineStr">
         <is>
-          <t>R S, 2025, J AM STAT ASSOC</t>
+          <t>Sun R, 2025, J AM STAT ASSOC</t>
         </is>
       </c>
     </row>

</xml_diff>